<commit_message>
Chico: 2022 versão 1
</commit_message>
<xml_diff>
--- a/bolao-max-server/json/Bolao.2022.xlsx
+++ b/bolao-max-server/json/Bolao.2022.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Dev\bolao.maxmat1.com.br\bolao-max-server\json\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F41267-5FBB-476E-BF56-9EEA73598F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA02C7B-B2EC-495D-A72E-9164763F9E3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="3" xr2:uid="{E832FB04-0F9E-4D5A-9979-8D7732736F4D}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="83">
   <si>
     <t>Nome</t>
   </si>
@@ -297,6 +297,18 @@
   </si>
   <si>
     <t>Fluminense</t>
+  </si>
+  <si>
+    <t>Chico 'Vírus'</t>
+  </si>
+  <si>
+    <t>Alan</t>
+  </si>
+  <si>
+    <t>Romulo</t>
+  </si>
+  <si>
+    <t>Daiane 'Pipoka'</t>
   </si>
 </sst>
 </file>
@@ -447,17 +459,26 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="32">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -471,15 +492,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -736,7 +748,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1020866</xdr:colOff>
+      <xdr:colOff>1020867</xdr:colOff>
       <xdr:row>61</xdr:row>
       <xdr:rowOff>34253</xdr:rowOff>
     </xdr:to>
@@ -763,6 +775,146 @@
         <a:xfrm>
           <a:off x="5992091" y="6734047"/>
           <a:ext cx="4709639" cy="4920706"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4097" name="AutoShape 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15081A12-8F75-4010-85AA-BB820D77F33F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12134850" y="7048500"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4098" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6AE6AF2E-8D68-4150-8EE0-2E638C63FF20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11010900" y="6858000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>297006</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>69273</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>470817</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>137506</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3ABEC4A4-5101-486B-8024-3A1DFDB453D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="297006" y="6736773"/>
+          <a:ext cx="4537993" cy="8069233"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -884,11 +1036,11 @@
   <autoFilter ref="A4:F34" xr:uid="{F5A25D63-F912-44E0-8847-35DF47A06A02}"/>
   <tableColumns count="6">
     <tableColumn id="2" xr3:uid="{FBFBCB0B-E6B9-472A-BBF4-8AFDF445D6B3}" uniqueName="2" name="N" queryTableFieldId="9" dataDxfId="5"/>
-    <tableColumn id="1" xr3:uid="{966EE970-706A-46DE-B74E-0913A5C56C2D}" uniqueName="1" name="Nome" queryTableFieldId="1" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{B66F3C6E-9BFA-4B66-8A32-938EB69221FB}" uniqueName="4" name="GP1" queryTableFieldId="4" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{2EF327B3-6F9C-4968-A886-2A34E87C9490}" uniqueName="5" name="GP2" queryTableFieldId="5" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{F4757D4D-A438-41D3-AF95-2D413C16752B}" uniqueName="6" name="GP3" queryTableFieldId="6" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{3D69F0C1-06FF-4832-BDC1-BD98097A4CA3}" uniqueName="7" name="GP4" queryTableFieldId="7" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{966EE970-706A-46DE-B74E-0913A5C56C2D}" uniqueName="1" name="Nome" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{B66F3C6E-9BFA-4B66-8A32-938EB69221FB}" uniqueName="4" name="GP1" queryTableFieldId="4" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{2EF327B3-6F9C-4968-A886-2A34E87C9490}" uniqueName="5" name="GP2" queryTableFieldId="5" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{F4757D4D-A438-41D3-AF95-2D413C16752B}" uniqueName="6" name="GP3" queryTableFieldId="6" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{3D69F0C1-06FF-4832-BDC1-BD98097A4CA3}" uniqueName="7" name="GP4" queryTableFieldId="7" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1267,27 +1419,27 @@
       <c r="F3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N3" s="13" t="s">
+      <c r="N3" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="O3" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="P3" s="13" t="s">
+      <c r="P3" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="Q3" s="13" t="s">
+      <c r="Q3" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="R3" s="13" t="s">
+      <c r="R3" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="S3" s="13" t="s">
+      <c r="S3" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1308,11 +1460,11 @@
       <c r="F4" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
       <c r="S4" s="2" t="s">
         <v>2</v>
       </c>
@@ -2808,10 +2960,10 @@
       <c r="F3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
+      <c r="S3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -5220,7 +5372,7 @@
   <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -5268,11 +5420,10 @@
       <c r="A5" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 1</v>
-      </c>
-      <c r="C5" s="14" t="s">
+      <c r="B5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -5287,19 +5438,18 @@
       <c r="G5"/>
       <c r="H5" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 1","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Carol","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B6" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 2</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>5</v>
+      <c r="B6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>17</v>
@@ -5313,19 +5463,18 @@
       <c r="G6"/>
       <c r="H6" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 2","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Guilherme","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 3</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>11</v>
+      <c r="B7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>5</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>14</v>
@@ -5339,19 +5488,18 @@
       <c r="G7"/>
       <c r="H7" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 3","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Chico 'Vírus'","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>4</v>
       </c>
-      <c r="B8" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 4</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>5</v>
+      <c r="B8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>78</v>
@@ -5365,18 +5513,17 @@
       <c r="G8"/>
       <c r="H8" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 4","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Leandro","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>5</v>
       </c>
-      <c r="B9" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 5</v>
-      </c>
-      <c r="C9" s="14" t="s">
+      <c r="B9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -5391,19 +5538,18 @@
       <c r="G9"/>
       <c r="H9" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 5","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Giovanni","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Goiás","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>6</v>
       </c>
-      <c r="B10" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 6</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>5</v>
+      <c r="B10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>23</v>
@@ -5417,18 +5563,17 @@
       <c r="G10"/>
       <c r="H10" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 6","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Gilson","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>7</v>
       </c>
-      <c r="B11" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 7</v>
-      </c>
-      <c r="C11" s="14" t="s">
+      <c r="B11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -5443,19 +5588,18 @@
       <c r="G11"/>
       <c r="H11" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 7","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Midão","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>8</v>
       </c>
-      <c r="B12" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 8</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>5</v>
+      <c r="B12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>17</v>
@@ -5469,18 +5613,17 @@
       <c r="G12"/>
       <c r="H12" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 8","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Fatinha","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>9</v>
       </c>
-      <c r="B13" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 9</v>
-      </c>
-      <c r="C13" s="14" t="s">
+      <c r="B13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -5495,18 +5638,17 @@
       <c r="G13"/>
       <c r="H13" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 9","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Miguel","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>10</v>
       </c>
-      <c r="B14" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 10</v>
-      </c>
-      <c r="C14" s="14" t="s">
+      <c r="B14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -5521,19 +5663,18 @@
       <c r="G14"/>
       <c r="H14" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 10","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Daiane 'Pipoka'","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>11</v>
       </c>
-      <c r="B15" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 11</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>11</v>
+      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>71</v>
@@ -5547,19 +5688,18 @@
       <c r="G15"/>
       <c r="H15" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 11","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Adriel","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>12</v>
       </c>
-      <c r="B16" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 12</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>5</v>
+      <c r="B16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>23</v>
@@ -5573,18 +5713,17 @@
       <c r="G16"/>
       <c r="H16" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 12","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Sérgio","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Botafogo","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>13</v>
       </c>
-      <c r="B17" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 13</v>
-      </c>
-      <c r="C17" s="14" t="s">
+      <c r="B17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -5599,19 +5738,18 @@
       <c r="G17"/>
       <c r="H17" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 13","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Max","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>14</v>
       </c>
-      <c r="B18" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 14</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>5</v>
+      <c r="B18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>17</v>
@@ -5625,18 +5763,17 @@
       <c r="G18"/>
       <c r="H18" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 14","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Terezinha","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>15</v>
       </c>
-      <c r="B19" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 15</v>
-      </c>
-      <c r="C19" s="14" t="s">
+      <c r="B19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -5651,19 +5788,18 @@
       <c r="G19"/>
       <c r="H19" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 15","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Geovane","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>16</v>
       </c>
-      <c r="B20" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 16</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>5</v>
+      <c r="B20" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>78</v>
@@ -5677,18 +5813,17 @@
       <c r="G20"/>
       <c r="H20" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 16","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Valdécio","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>17</v>
       </c>
-      <c r="B21" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 17</v>
-      </c>
-      <c r="C21" s="14" t="s">
+      <c r="B21" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -5703,19 +5838,18 @@
       <c r="G21"/>
       <c r="H21" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 17","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Chamon","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Coritiba","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>18</v>
       </c>
-      <c r="B22" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 18</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>5</v>
+      <c r="B22" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>23</v>
@@ -5729,19 +5863,18 @@
       <c r="G22"/>
       <c r="H22" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 18","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Alan","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>19</v>
       </c>
-      <c r="B23" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 19</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>11</v>
+      <c r="B23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>13</v>
@@ -5755,19 +5888,18 @@
       <c r="G23"/>
       <c r="H23" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 19","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Wagner","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>20</v>
       </c>
-      <c r="B24" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 20</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>5</v>
+      <c r="B24" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>17</v>
@@ -5781,18 +5913,17 @@
       <c r="G24"/>
       <c r="H24" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 20","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Tiago","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>21</v>
       </c>
-      <c r="B25" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 21</v>
-      </c>
-      <c r="C25" s="14" t="s">
+      <c r="B25" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -5807,19 +5938,18 @@
       <c r="G25"/>
       <c r="H25" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 21","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Romulo","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>22</v>
       </c>
-      <c r="B26" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 22</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>5</v>
+      <c r="B26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>78</v>
@@ -5833,18 +5963,17 @@
       <c r="G26"/>
       <c r="H26" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 22","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Renato","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>23</v>
       </c>
-      <c r="B27" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 23</v>
-      </c>
-      <c r="C27" s="14" t="s">
+      <c r="B27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -5859,19 +5988,18 @@
       <c r="G27"/>
       <c r="H27" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 23","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Willian","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>24</v>
       </c>
-      <c r="B28" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 24</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>5</v>
+      <c r="B28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>23</v>
@@ -5885,19 +6013,18 @@
       <c r="G28"/>
       <c r="H28" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 24","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Ana Cristina","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>25</v>
       </c>
-      <c r="B29" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 25</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>11</v>
+      <c r="B29" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>13</v>
@@ -5911,19 +6038,18 @@
       <c r="G29"/>
       <c r="H29" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 25","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Marlon","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Corinthians","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Juventude","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>26</v>
       </c>
-      <c r="B30" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 26</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>5</v>
+      <c r="B30" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>17</v>
@@ -5937,18 +6063,17 @@
       <c r="G30"/>
       <c r="H30" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 26","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Deca","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fortaleza","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Ceará","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>27</v>
       </c>
-      <c r="B31" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 27</v>
-      </c>
-      <c r="C31" s="14" t="s">
+      <c r="B31" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -5963,19 +6088,18 @@
       <c r="G31"/>
       <c r="H31" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 27","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Marilda","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Bragantino","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Santos","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Avaí","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>28</v>
       </c>
-      <c r="B32" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 28</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>5</v>
+      <c r="B32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>78</v>
@@ -5989,18 +6113,17 @@
       <c r="G32"/>
       <c r="H32" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 28","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Anna Maria","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Fluminense","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Internacional","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>29</v>
       </c>
-      <c r="B33" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 29</v>
-      </c>
-      <c r="C33" s="14" t="s">
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -6015,19 +6138,18 @@
       <c r="G33"/>
       <c r="H33" t="str">
         <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 29","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <v>{"Nome": "Jean","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Flamengo","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "América-MG","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "São Paulo","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>30</v>
       </c>
-      <c r="B34" s="1" t="str">
-        <f>"Boleiro "&amp;bolao345[[#This Row],[N]]</f>
-        <v>Boleiro 30</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>5</v>
+      <c r="B34" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>23</v>
@@ -6040,8 +6162,8 @@
       </c>
       <c r="G34"/>
       <c r="H34" t="str">
-        <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]},"</f>
-        <v>{"Nome": "Boleiro 30","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Palmeiras","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]},</v>
+        <f>"{""Nome"": """&amp;bolao345[[#This Row],[Nome]]&amp;""",""Pontos"": 0,""Saldo_Gols"": 0,""golsPro"": 0,""Posicao"": 0,""Premio"": 1, ""Clubes"": [{""Grupo"": ""GP1"",""Clube"": """&amp;bolao345[[#This Row],[GP1]]&amp;""",""pontos"": ""9"",""jogos"": ""8"",""vitorias"": ""3"",""empates"": ""0"",""derrotas"": ""5"",""golsPro"": ""11"",""golsContra"": ""13"",""saldoGols"": ""-2"",""percentual"": ""37.5"",""Coracao"": false},{""Grupo"": ""GP2"",""Clube"": """&amp;bolao345[[#This Row],[GP2]]&amp;""",""pontos"": ""20"",""jogos"": ""9"",""vitorias"": ""6"",""empates"": ""2"",""derrotas"": ""1"",""golsPro"": ""16"",""golsContra"": ""6"",""saldoGols"": ""10"",""percentual"": ""74.1"",""Coracao"": false},{""Grupo"": ""GP3"",""Clube"": """&amp;bolao345[[#This Row],[GP3]]&amp;""",""pontos"": ""10"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""4"",""derrotas"": ""3"",""golsPro"": ""12"",""golsContra"": ""18"",""saldoGols"": ""-6"",""percentual"": ""37.0"",""Coracao"": false},{""Grupo"": ""GP4"",""Clube"": """&amp;bolao345[[#This Row],[GP4]]&amp;""",""pontos"": ""8"",""jogos"": ""9"",""vitorias"": ""2"",""empates"": ""2"",""derrotas"": ""5"",""golsPro"": ""15"",""golsContra"": ""20"",""saldoGols"": ""-5"",""percentual"": ""29.6"",""Coracao"": false}]}"</f>
+        <v>{"Nome": "Eduardo","Pontos": 0,"Saldo_Gols": 0,"golsPro": 0,"Posicao": 0,"Premio": 1, "Clubes": [{"Grupo": "GP1","Clube": "Atlético-MG","pontos": "9","jogos": "8","vitorias": "3","empates": "0","derrotas": "5","golsPro": "11","golsContra": "13","saldoGols": "-2","percentual": "37.5","Coracao": false},{"Grupo": "GP2","Clube": "Atlético-GO","pontos": "20","jogos": "9","vitorias": "6","empates": "2","derrotas": "1","golsPro": "16","golsContra": "6","saldoGols": "10","percentual": "74.1","Coracao": false},{"Grupo": "GP3","Clube": "Athletico-PR","pontos": "10","jogos": "9","vitorias": "2","empates": "4","derrotas": "3","golsPro": "12","golsContra": "18","saldoGols": "-6","percentual": "37.0","Coracao": false},{"Grupo": "GP4","Clube": "Cuiabá","pontos": "8","jogos": "9","vitorias": "2","empates": "2","derrotas": "5","golsPro": "15","golsContra": "20","saldoGols": "-5","percentual": "29.6","Coracao": false}]}</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>